<commit_message>
fix: refine excel import and export review labels
</commit_message>
<xml_diff>
--- a/templates/笔记导入模板.xlsx
+++ b/templates/笔记导入模板.xlsx
@@ -4,15 +4,14 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="5" rupBuild="9303"/>
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
-    <sheet sheetId="1" name="笔记导入" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="填写说明" state="visible" r:id="rId5"/>
+    <sheet sheetId="1" name="笔记导入模板" state="visible" r:id="rId4"/>
   </sheets>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
   <si>
     <t>平台（必填）</t>
   </si>
@@ -29,7 +28,7 @@
     <t>阶段（IFFO/GUM）</t>
   </si>
   <si>
-    <t>订单编号（必填）</t>
+    <t>订单编号</t>
   </si>
   <si>
     <t>内容渠道（必填）</t>
@@ -50,7 +49,7 @@
     <t>示例客户</t>
   </si>
   <si>
-    <t>爱他美澳洲白金版</t>
+    <t>爱他美奇迹绿罐</t>
   </si>
   <si>
     <t>IFFO</t>
@@ -61,120 +60,6 @@
   <si>
     <t>https://xhslink.com/示例短链</t>
   </si>
-  <si>
-    <t>标准字段</t>
-  </si>
-  <si>
-    <t>显示名称</t>
-  </si>
-  <si>
-    <t>是否必填</t>
-  </si>
-  <si>
-    <t>字段说明</t>
-  </si>
-  <si>
-    <t>支持别名</t>
-  </si>
-  <si>
-    <t>模板版本</t>
-  </si>
-  <si>
-    <t>template-2026.07.30.1</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>模板Schema 1</t>
-  </si>
-  <si>
-    <t>模板随审核规则同步更新</t>
-  </si>
-  <si>
-    <t>platform</t>
-  </si>
-  <si>
-    <t>是</t>
-  </si>
-  <si>
-    <t>线下表格的平台标识，仅用于记录和导出</t>
-  </si>
-  <si>
-    <t>平台、平台（必填）、所属平台、platform</t>
-  </si>
-  <si>
-    <t>shopName</t>
-  </si>
-  <si>
-    <t>线下表格中的店铺名称，仅用于记录和导出</t>
-  </si>
-  <si>
-    <t>店铺名称、店铺名称（必填）、店铺、shopName</t>
-  </si>
-  <si>
-    <t>customerName</t>
-  </si>
-  <si>
-    <t>线下表格中的客户名，仅用于记录和导出</t>
-  </si>
-  <si>
-    <t>客户名、客户名（必填）、客户名称、customerName</t>
-  </si>
-  <si>
-    <t>productName</t>
-  </si>
-  <si>
-    <t>系统中已有的产品名称、产品系列或简称</t>
-  </si>
-  <si>
-    <t>产品、产品系列、产品系列（必填）、商品、商品名称、产品名称、审核产品、product、productName</t>
-  </si>
-  <si>
-    <t>productStage</t>
-  </si>
-  <si>
-    <t>必填，只填写 IFFO 或 GUM</t>
-  </si>
-  <si>
-    <t>产品阶段话题、产品段位、奶粉段位、阶段、阶段（IFFO/GUM）、段位、productStage</t>
-  </si>
-  <si>
-    <t>orderNumber</t>
-  </si>
-  <si>
-    <t>用于和原始表格对照，不参与审核判断</t>
-  </si>
-  <si>
-    <t>订单编号、订单号、订单编号（必填）、orderNumber</t>
-  </si>
-  <si>
-    <t>contentChannel</t>
-  </si>
-  <si>
-    <t>原表中的内容渠道；不会扩展当前审核引擎能力</t>
-  </si>
-  <si>
-    <t>内容渠道、内容渠道（必填）、发布渠道、内容平台、channel</t>
-  </si>
-  <si>
-    <t>noteUrl</t>
-  </si>
-  <si>
-    <t>小红书完整链接或 xhslink 短链接</t>
-  </si>
-  <si>
-    <t>笔记链接、小红书链接、链接、链接（必填）、文章链接、笔记地址、小红书笔记链接、noteUrl、url、link</t>
-  </si>
-  <si>
-    <t>publishTime</t>
-  </si>
-  <si>
-    <t>线下表格中的发帖时间，仅用于记录和导出</t>
-  </si>
-  <si>
-    <t>发帖时间、发帖时间（必填）、发布时间、发布日期、笔记时间、publishTime、createdAt</t>
-  </si>
 </sst>
 </file>
 
@@ -183,7 +68,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd hh:mm:ss"/>
   </numFmts>
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <color theme="1"/>
       <family val="2"/>
@@ -194,9 +79,6 @@
     <font>
       <b/>
       <color rgb="FF000000"/>
-    </font>
-    <font>
-      <b/>
     </font>
   </fonts>
   <fills count="3">
@@ -224,7 +106,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -233,13 +115,9 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -586,14 +464,14 @@
     <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="3" width="20" customWidth="1"/>
     <col min="4" max="4" width="26" customWidth="1"/>
-    <col min="5" max="5" width="12" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
     <col min="6" max="6" width="22" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
     <col min="8" max="8" width="52" style="1" customWidth="1"/>
     <col min="9" max="9" width="22" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" s="3" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -615,10 +493,10 @@
       <c r="G1" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="4" t="s">
+      <c r="H1" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="5" t="s">
+      <c r="I1" s="4" t="s">
         <v>8</v>
       </c>
     </row>
@@ -5651,7 +5529,7 @@
     <row r="5000" spans="5:5" x14ac:dyDescent="0.25"/>
     <row r="5001" spans="5:5" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <autoFilter ref="A1:I5001"/>
+  <autoFilter ref="A1:I1"/>
   <dataValidations count="2">
     <dataValidation type="list" showErrorMessage="1" errorTitle="产品阶段话题无效" error="产品阶段话题请填写 IFFO 或 GUM。" sqref="E10:E5001">
       <formula1>"IFFO,GUM"</formula1>
@@ -5663,209 +5541,4 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E11"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <cols>
-    <col min="1" max="1" width="22" customWidth="1"/>
-    <col min="2" max="2" width="20" customWidth="1"/>
-    <col min="3" max="3" width="12" customWidth="1"/>
-    <col min="4" max="4" width="48" customWidth="1"/>
-    <col min="5" max="5" width="72" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="6" t="s">
-        <v>16</v>
-      </c>
-      <c r="B1" s="6" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D1" s="6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E1" s="6" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" t="s">
-        <v>0</v>
-      </c>
-      <c r="C3" t="s">
-        <v>27</v>
-      </c>
-      <c r="D3" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B4" t="s">
-        <v>1</v>
-      </c>
-      <c r="C4" t="s">
-        <v>27</v>
-      </c>
-      <c r="D4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E4" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>33</v>
-      </c>
-      <c r="B5" t="s">
-        <v>2</v>
-      </c>
-      <c r="C5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D5" t="s">
-        <v>34</v>
-      </c>
-      <c r="E5" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>36</v>
-      </c>
-      <c r="B6" t="s">
-        <v>3</v>
-      </c>
-      <c r="C6" t="s">
-        <v>27</v>
-      </c>
-      <c r="D6" t="s">
-        <v>37</v>
-      </c>
-      <c r="E6" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>39</v>
-      </c>
-      <c r="B7" t="s">
-        <v>4</v>
-      </c>
-      <c r="C7" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" t="s">
-        <v>40</v>
-      </c>
-      <c r="E7" t="s">
-        <v>41</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>42</v>
-      </c>
-      <c r="B8" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" t="s">
-        <v>27</v>
-      </c>
-      <c r="D8" t="s">
-        <v>43</v>
-      </c>
-      <c r="E8" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>45</v>
-      </c>
-      <c r="B9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>48</v>
-      </c>
-      <c r="B10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C10" t="s">
-        <v>27</v>
-      </c>
-      <c r="D10" t="s">
-        <v>49</v>
-      </c>
-      <c r="E10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>51</v>
-      </c>
-      <c r="B11" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" t="s">
-        <v>27</v>
-      </c>
-      <c r="D11" t="s">
-        <v>52</v>
-      </c>
-      <c r="E11" t="s">
-        <v>53</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
fix: separate store aliases and stage fields
</commit_message>
<xml_diff>
--- a/templates/笔记导入模板.xlsx
+++ b/templates/笔记导入模板.xlsx
@@ -5,19 +5,15 @@
   <workbookPr defaultThemeVersion="164011" filterPrivacy="1"/>
   <sheets>
     <sheet sheetId="1" name="达能客户导入" state="visible" r:id="rId4"/>
-    <sheet sheetId="2" name="活动列表" state="veryHidden" r:id="rId5"/>
-    <sheet sheetId="3" name="填写说明" state="visible" r:id="rId6"/>
-    <sheet sheetId="4" name="VERIDIA模板信息" state="veryHidden" r:id="rId7"/>
+    <sheet sheetId="2" name="填写说明" state="visible" r:id="rId5"/>
+    <sheet sheetId="3" name="VERIDIA模板信息" state="veryHidden" r:id="rId6"/>
   </sheets>
-  <definedNames>
-    <definedName name="VERIDIA_ACTIVITY_NAMES">'活动列表'!$A$2:$A$7</definedName>
-  </definedNames>
   <calcPr calcId="171027"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="86">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="78">
   <si>
     <t>平台（必填）</t>
   </si>
@@ -31,12 +27,12 @@
     <t>产品系列（必填）</t>
   </si>
   <si>
+    <t>段位（必填）</t>
+  </si>
+  <si>
     <t>阶段（必填）</t>
   </si>
   <si>
-    <t>段位（必填）</t>
-  </si>
-  <si>
     <t>订单编号（必填）</t>
   </si>
   <si>
@@ -79,31 +75,7 @@
     <t>https://xhslink.com/示例短链</t>
   </si>
   <si>
-    <t>佳贝艾特2026年8月小红书种草审核</t>
-  </si>
-  <si>
-    <t>活动名称</t>
-  </si>
-  <si>
-    <t>内容渠道</t>
-  </si>
-  <si>
-    <t>佳贝艾特2026年8月抖音种草审核</t>
-  </si>
-  <si>
-    <t>抖音</t>
-  </si>
-  <si>
-    <t>爱他美2026年8月小红书种草审核</t>
-  </si>
-  <si>
-    <t>爱他美2026年8月抖音种草审核</t>
-  </si>
-  <si>
-    <t>爱他美2026年7月小红书种草审核</t>
-  </si>
-  <si>
-    <t>爱他美2026年7月抖音种草审核</t>
+    <t/>
   </si>
   <si>
     <t>标准字段</t>
@@ -127,9 +99,6 @@
     <t>template-2026.08.07.1</t>
   </si>
   <si>
-    <t/>
-  </si>
-  <si>
     <t>模板Schema 1</t>
   </si>
   <si>
@@ -155,6 +124,9 @@
   </si>
   <si>
     <t>活动请选择完整的抖音审核活动名称；链接支持 https://www.douyin.com/note/...、https://www.douyin.com/video/... 或 https://v.douyin.com/...。</t>
+  </si>
+  <si>
+    <t>XXX2026年8月抖音种草审核</t>
   </si>
   <si>
     <t>模板类型</t>
@@ -768,18 +740,15 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:K2"/>
-  <dataValidations count="4">
-    <dataValidation type="list" showErrorMessage="1" errorTitle="阶段无效" error="阶段请填写 P段、1段、2段、3段、4段、1+或2+。" sqref="E2:E5001">
+  <dataValidations count="3">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="段位无效" error="段位请填写 P段、1段、2段、3段、4段、1+或2+。" sqref="E2:E5001">
       <formula1>"P段,1段,2段,3段,4段,1+段,2+段"</formula1>
     </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="段位无效" error="段位仅支持 IFFO 或 GUM" sqref="F2:F5001">
+    <dataValidation type="list" showErrorMessage="1" errorTitle="阶段无效" error="阶段仅支持 IFFO 或 GUM" sqref="F2:F5001">
       <formula1>"IFFO,GUM"</formula1>
     </dataValidation>
     <dataValidation type="list" showErrorMessage="1" errorTitle="内容渠道无效" error="内容渠道仅支持小红书或抖音，并且必须与活动及链接一致。" sqref="H2:H10000">
       <formula1>"小红书,抖音"</formula1>
-    </dataValidation>
-    <dataValidation type="list" showErrorMessage="1" errorTitle="活动名称无效" error="请选择活动管理中当前启用的完整活动名称。" sqref="K2:K10000">
-      <formula1>VERIDIA_ACTIVITY_NAMES</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -788,73 +757,6 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
-  <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" t="s">
-        <v>21</v>
-      </c>
-      <c r="B1" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>20</v>
-      </c>
-      <c r="B2" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B3" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>25</v>
-      </c>
-      <c r="B4" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>26</v>
-      </c>
-      <c r="B5" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>27</v>
-      </c>
-      <c r="B6" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>28</v>
-      </c>
-      <c r="B7" t="s">
-        <v>24</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E16"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
@@ -868,274 +770,274 @@
   <sheetData>
     <row r="1" spans="1:5" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="6" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="B1" s="6" t="s">
-        <v>30</v>
+        <v>22</v>
       </c>
       <c r="C1" s="6" t="s">
-        <v>31</v>
+        <v>23</v>
       </c>
       <c r="D1" s="6" t="s">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="E1" s="6" t="s">
-        <v>33</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
       <c r="C2" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D2" t="s">
-        <v>37</v>
+        <v>28</v>
       </c>
       <c r="E2" t="s">
-        <v>38</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>39</v>
+        <v>30</v>
       </c>
       <c r="B3" t="s">
         <v>10</v>
       </c>
       <c r="C3" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="E3" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
         <v>36</v>
       </c>
-      <c r="D4" t="s">
-        <v>45</v>
-      </c>
       <c r="E4" t="s">
-        <v>23</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>46</v>
+        <v>38</v>
       </c>
       <c r="B5" t="s">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="C5" t="s">
-        <v>36</v>
+        <v>20</v>
       </c>
       <c r="D5" t="s">
-        <v>48</v>
+        <v>40</v>
       </c>
       <c r="E5" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>42</v>
       </c>
       <c r="B6" t="s">
         <v>0</v>
       </c>
       <c r="C6" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>51</v>
+        <v>43</v>
       </c>
       <c r="E6" t="s">
-        <v>52</v>
+        <v>44</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="B7" t="s">
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D7" t="s">
-        <v>54</v>
+        <v>46</v>
       </c>
       <c r="E7" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>56</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
         <v>2</v>
       </c>
       <c r="C8" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E8" t="s">
-        <v>58</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>59</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
         <v>3</v>
       </c>
       <c r="C9" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D9" t="s">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>53</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>62</v>
+        <v>54</v>
       </c>
       <c r="B10" t="s">
         <v>4</v>
       </c>
       <c r="C10" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D10" t="s">
-        <v>63</v>
+        <v>55</v>
       </c>
       <c r="E10" t="s">
-        <v>64</v>
+        <v>56</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>65</v>
+        <v>57</v>
       </c>
       <c r="B11" t="s">
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D11" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
       <c r="E11" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
       <c r="B12" t="s">
         <v>6</v>
       </c>
       <c r="C12" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D12" t="s">
-        <v>69</v>
+        <v>61</v>
       </c>
       <c r="E12" t="s">
-        <v>70</v>
+        <v>62</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>71</v>
+        <v>63</v>
       </c>
       <c r="B13" t="s">
         <v>7</v>
       </c>
       <c r="C13" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D13" t="s">
-        <v>72</v>
+        <v>64</v>
       </c>
       <c r="E13" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="B14" t="s">
         <v>8</v>
       </c>
       <c r="C14" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D14" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="E14" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="B15" t="s">
         <v>9</v>
       </c>
       <c r="C15" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D15" t="s">
-        <v>78</v>
+        <v>70</v>
       </c>
       <c r="E15" t="s">
-        <v>79</v>
+        <v>71</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>80</v>
+        <v>72</v>
       </c>
       <c r="B16" t="s">
         <v>10</v>
       </c>
       <c r="C16" t="s">
-        <v>40</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>81</v>
+        <v>73</v>
       </c>
       <c r="E16" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>
@@ -1144,25 +1046,25 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:B2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>83</v>
+        <v>75</v>
       </c>
       <c r="B1" t="s">
-        <v>84</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>85</v>
+        <v>77</v>
       </c>
       <c r="B2" t="s">
-        <v>35</v>
+        <v>27</v>
       </c>
     </row>
   </sheetData>

</xml_diff>